<commit_message>
merge: fixes from advisors and data room improvments
</commit_message>
<xml_diff>
--- a/dataroom/1_company_fundamentals/1.4_investment_docs/ecentic-cap-table.xlsx
+++ b/dataroom/1_company_fundamentals/1.4_investment_docs/ecentic-cap-table.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Cap Table" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Round Scenarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="€500K Round Scenarios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vesting Schedule" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -121,12 +121,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,9 +142,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -524,7 +521,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,14 +534,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As of 2 June 2026 · Pre-money, prior to any external financing</t>
+          <t>As of 2 June 2026 · Pre-money, prior to €500K seed</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Authorized share capital: 100,000 Common Shares · Par value: 1 ALL · Total registered capital: 100,000 ALL</t>
+          <t>Authorized: 100,000 Common Shares · Par: 1 ALL · Registered capital: 100,000 ALL</t>
         </is>
       </c>
     </row>
@@ -571,12 +568,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>% Issued (Today)</t>
+          <t>% Issued</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>% Fully Diluted (post-ESOP)</t>
+          <t>% Fully Diluted</t>
         </is>
       </c>
     </row>
@@ -616,7 +613,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Founder · CTO</t>
+          <t>Founder · CDO</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -691,16 +688,8 @@
           <t>ESOP Pool (reserved, unissued)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Reserved</t>
-        </is>
-      </c>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
       <c r="D10" s="11" t="n">
         <v>11111</v>
       </c>
@@ -724,7 +713,7 @@
         <f>D9+D10</f>
         <v/>
       </c>
-      <c r="E11" s="9" t="inlineStr"/>
+      <c r="E11" s="7" t="n"/>
       <c r="F11" s="9" t="n">
         <v>1</v>
       </c>
@@ -739,28 +728,28 @@
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>1. All Common Shares are subject to 4-year vesting with 1-year cliff, with vesting Start Date being the date of incorporation per the Shareholders Agreement.</t>
+          <t>1. All Common Shares subject to 4-year vesting with 1-year cliff. Vesting Start Date = date of incorporation.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>2. ESOP Pool is reserved as authorized-but-unissued capacity (11,111 shares) representing 10% of fully diluted capital. Shares issued upon Option exercise will require a share capital increase by shareholder resolution.</t>
+          <t>2. ESOP Pool reserved as authorized-but-unissued capacity (11,111 shares = 10% fully diluted). Issued upon grant + share capital increase.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>3. Mario Vukzaj (Product) and Arbi Kullakshi (AI) currently engage with the Company as independent contractors with no equity stake and no Options granted as of this date.</t>
+          <t>3. Two contractors (Design freelancer + AI freelancer) hold no equity and no Options.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>4. Founders' email aliases: firstname.lastname@ecentic.ai</t>
+          <t>4. Founder email aliases: firstname@ecentic.ai</t>
         </is>
       </c>
     </row>
@@ -784,7 +773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -796,7 +785,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>€300K Round — Post-Money Scenarios</t>
+          <t>€500K Seed Round — Post-Money Scenarios</t>
         </is>
       </c>
     </row>
@@ -822,7 +811,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>€300,000</t>
+          <t>€500,000</t>
         </is>
       </c>
     </row>
@@ -870,81 +859,81 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr"/>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Scenario A (€3M post)</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>Scenario B (€4M post)</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>Scenario C (€5M post)</t>
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Scenario A (€4M post)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Scenario B (€5M post)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Scenario C (€6M post)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Post-money valuation</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="C13" s="18" t="n">
+      <c r="B13" s="17" t="n">
         <v>4000000</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="C13" s="17" t="n">
         <v>5000000</v>
       </c>
+      <c r="D13" s="17" t="n">
+        <v>6000000</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Pre-money valuation</t>
         </is>
       </c>
-      <c r="B14" s="18">
-        <f>B13-300000</f>
-        <v/>
-      </c>
-      <c r="C14" s="18">
-        <f>C13-300000</f>
-        <v/>
-      </c>
-      <c r="D14" s="18">
-        <f>D13-300000</f>
+      <c r="B14" s="17">
+        <f>B13-500000</f>
+        <v/>
+      </c>
+      <c r="C14" s="17">
+        <f>C13-500000</f>
+        <v/>
+      </c>
+      <c r="D14" s="17">
+        <f>D13-500000</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Investor ownership %</t>
         </is>
       </c>
       <c r="B15" s="6">
-        <f>300000/B13</f>
+        <f>500000/B13</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>300000/C13</f>
+        <f>500000/C13</f>
         <v/>
       </c>
       <c r="D15" s="6">
-        <f>300000/D13</f>
+        <f>500000/D13</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Founders' combined ownership % (post-round, post-ESOP)</t>
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Founders combined % (post-round, post-ESOP)</t>
         </is>
       </c>
       <c r="B16" s="6">
@@ -961,9 +950,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>Xhurian Shaba (40% founder share) — post-round %</t>
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>Xhurian (40% founder share) — post-round %</t>
         </is>
       </c>
       <c r="B17" s="6">
@@ -980,9 +969,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>Alvi Palloshi (30% founder share) — post-round %</t>
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>Alvi (30% founder share) — post-round %</t>
         </is>
       </c>
       <c r="B18" s="6">
@@ -999,9 +988,9 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Iseld Muça (30% founder share) — post-round %</t>
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>Iseld (30% founder share) — post-round %</t>
         </is>
       </c>
       <c r="B19" s="6">
@@ -1018,7 +1007,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>ESOP — post-round %</t>
         </is>
@@ -1037,20 +1026,20 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Sanity check (sum = 100%)</t>
         </is>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="20">
         <f>B15+B16+B20</f>
         <v/>
       </c>
-      <c r="C21" s="21">
+      <c r="C21" s="20">
         <f>C15+C16+C20</f>
         <v/>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="20">
         <f>D15+D16+D20</f>
         <v/>
       </c>
@@ -1065,26 +1054,34 @@
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>1. Scenarios assume the ESOP pool is sized to 10% of post-round fully diluted capital. If sized pre-money, founders are diluted more; if sized post-money ("shuffle"), investor is diluted more. Default assumption here: post-round.</t>
+          <t>1. Scenarios assume ESOP pool sized to 10% of post-round fully diluted (post-money treatment — investor takes that dilution).</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>2. SAFEs (Simple Agreement for Future Equity) would convert at the post-money cap shown, less any standard discount or MFN protections negotiated.</t>
+          <t>2. €500K at €5M post = 10% investor ownership. Aligns with European pre-seed comparables for AI infrastructure / e-commerce SaaS with live revenue.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>3. Recommendation: target Scenario B (€4M post-money) for €300K SAFE = 7.5% investor ownership. Aligns with European pre-seed comparables for AI infrastructure / e-commerce SaaS.</t>
+          <t>3. Recommended anchor: Scenario B (€5M post-money). Range €4M–€6M is defensible given current traction (2 paying customers, App Store live, enterprise pipeline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>4. SAFE conversion: at post-money cap shown, less any standard discount / MFN protections negotiated.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="A25:D25"/>
@@ -1101,14 +1098,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1127,39 +1124,39 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Cumulative % Vested</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Xhurian (40K shares)</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>Alvi (30K shares)</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
-        <is>
-          <t>Iseld (30K shares)</t>
-        </is>
-      </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>% Vested</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Xhurian (40K)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Alvi (30K)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Iseld (30K)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="n">
+      <c r="A5" s="21" t="n">
         <v>0</v>
       </c>
       <c r="B5" s="6" t="n">
@@ -1179,12 +1176,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Incorporation. No vesting yet.</t>
+          <t>Incorporation. No vesting.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="n">
+      <c r="A6" s="21" t="n">
         <v>6</v>
       </c>
       <c r="B6" s="6" t="n">
@@ -1204,12 +1201,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Mid-cliff. Still 0% vested.</t>
+          <t>Mid-cliff. Still 0%.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="n">
+      <c r="A7" s="21" t="n">
         <v>12</v>
       </c>
       <c r="B7" s="6" t="n">
@@ -1229,12 +1226,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Cliff complete — 25% vests in one block.</t>
+          <t>Cliff — 25% vests in one block.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n">
+      <c r="A8" s="21" t="n">
         <v>18</v>
       </c>
       <c r="B8" s="6" t="n">
@@ -1254,12 +1251,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Linear monthly vesting begins after cliff.</t>
+          <t>Linear monthly vesting begins.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n">
+      <c r="A9" s="21" t="n">
         <v>24</v>
       </c>
       <c r="B9" s="6" t="n">
@@ -1284,7 +1281,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n">
+      <c r="A10" s="21" t="n">
         <v>36</v>
       </c>
       <c r="B10" s="6" t="n">
@@ -1309,7 +1306,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n">
+      <c r="A11" s="21" t="n">
         <v>48</v>
       </c>
       <c r="B11" s="6" t="n">
@@ -1333,41 +1330,10 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Acceleration Triggers (per Section 3.4 of Shareholders Agreement)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>• Double-trigger: 100% of unvested shares accelerate on a Change of Control IF the Founder is terminated without Cause OR resigns for Good Reason within 12 months following the transaction.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>• Death or Permanent Disability: pro-rata vesting up to the date of the event.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
-          <t>• Termination for Cause: all unvested shares are forfeited and subject to Company repurchase at par.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>